<commit_message>
chore(excel): update the company evaluation form template
</commit_message>
<xml_diff>
--- a/app/Excel/1. Evaluation Form.xlsx
+++ b/app/Excel/1. Evaluation Form.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr filterPrivacy="1" hidePivotFieldList="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C238BF97-1275-4A3A-8A23-B7687A407215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC7C48D4-5349-4A81-ACBA-C15A76A81F8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A6A0F9D7-1262-4376-8878-27E284A36841}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="57">
   <si>
     <t>Course Name :</t>
   </si>
@@ -247,6 +247,9 @@
   </si>
   <si>
     <t>Column19</t>
+  </si>
+  <si>
+    <t>Part 4 :</t>
   </si>
 </sst>
 </file>
@@ -2008,35 +2011,35 @@
     <xf numFmtId="0" fontId="15" fillId="3" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="47" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="190" fontId="28" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="189" fontId="65" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="66" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="61" fillId="8" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="190" fontId="28" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="65" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="189" fontId="65" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="66" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -10829,7 +10832,7 @@
       <c r="V8" s="198"/>
       <c r="W8" s="198"/>
       <c r="X8" s="197" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="Y8" s="196"/>
       <c r="Z8" s="195" t="s">
@@ -12378,24 +12381,24 @@
       <c r="AY3" s="49"/>
       <c r="AZ3" s="49"/>
       <c r="BA3" s="49"/>
-      <c r="BB3" s="207" t="str">
+      <c r="BB3" s="215" t="str">
         <f>'01-Database'!D3</f>
         <v>courseName</v>
       </c>
-      <c r="BC3" s="207"/>
-      <c r="BD3" s="207"/>
-      <c r="BE3" s="207"/>
-      <c r="BF3" s="207"/>
-      <c r="BG3" s="207"/>
-      <c r="BH3" s="207"/>
-      <c r="BI3" s="207"/>
-      <c r="BJ3" s="207"/>
-      <c r="BK3" s="207"/>
-      <c r="BL3" s="207"/>
-      <c r="BM3" s="207"/>
-      <c r="BN3" s="207"/>
-      <c r="BO3" s="207"/>
-      <c r="BP3" s="207"/>
+      <c r="BC3" s="215"/>
+      <c r="BD3" s="215"/>
+      <c r="BE3" s="215"/>
+      <c r="BF3" s="215"/>
+      <c r="BG3" s="215"/>
+      <c r="BH3" s="215"/>
+      <c r="BI3" s="215"/>
+      <c r="BJ3" s="215"/>
+      <c r="BK3" s="215"/>
+      <c r="BL3" s="215"/>
+      <c r="BM3" s="215"/>
+      <c r="BN3" s="215"/>
+      <c r="BO3" s="215"/>
+      <c r="BP3" s="215"/>
     </row>
     <row r="4" spans="1:70" ht="24.6">
       <c r="A4"/>
@@ -12423,21 +12426,21 @@
       <c r="AY4" s="49"/>
       <c r="AZ4" s="49"/>
       <c r="BA4" s="49"/>
-      <c r="BB4" s="207"/>
-      <c r="BC4" s="207"/>
-      <c r="BD4" s="207"/>
-      <c r="BE4" s="207"/>
-      <c r="BF4" s="207"/>
-      <c r="BG4" s="207"/>
-      <c r="BH4" s="207"/>
-      <c r="BI4" s="207"/>
-      <c r="BJ4" s="207"/>
-      <c r="BK4" s="207"/>
-      <c r="BL4" s="207"/>
-      <c r="BM4" s="207"/>
-      <c r="BN4" s="207"/>
-      <c r="BO4" s="207"/>
-      <c r="BP4" s="207"/>
+      <c r="BB4" s="215"/>
+      <c r="BC4" s="215"/>
+      <c r="BD4" s="215"/>
+      <c r="BE4" s="215"/>
+      <c r="BF4" s="215"/>
+      <c r="BG4" s="215"/>
+      <c r="BH4" s="215"/>
+      <c r="BI4" s="215"/>
+      <c r="BJ4" s="215"/>
+      <c r="BK4" s="215"/>
+      <c r="BL4" s="215"/>
+      <c r="BM4" s="215"/>
+      <c r="BN4" s="215"/>
+      <c r="BO4" s="215"/>
+      <c r="BP4" s="215"/>
     </row>
     <row r="5" spans="1:70">
       <c r="A5"/>
@@ -12465,21 +12468,21 @@
       <c r="AY5" s="49"/>
       <c r="AZ5" s="49"/>
       <c r="BA5" s="49"/>
-      <c r="BB5" s="207"/>
-      <c r="BC5" s="207"/>
-      <c r="BD5" s="207"/>
-      <c r="BE5" s="207"/>
-      <c r="BF5" s="207"/>
-      <c r="BG5" s="207"/>
-      <c r="BH5" s="207"/>
-      <c r="BI5" s="207"/>
-      <c r="BJ5" s="207"/>
-      <c r="BK5" s="207"/>
-      <c r="BL5" s="207"/>
-      <c r="BM5" s="207"/>
-      <c r="BN5" s="207"/>
-      <c r="BO5" s="207"/>
-      <c r="BP5" s="207"/>
+      <c r="BB5" s="215"/>
+      <c r="BC5" s="215"/>
+      <c r="BD5" s="215"/>
+      <c r="BE5" s="215"/>
+      <c r="BF5" s="215"/>
+      <c r="BG5" s="215"/>
+      <c r="BH5" s="215"/>
+      <c r="BI5" s="215"/>
+      <c r="BJ5" s="215"/>
+      <c r="BK5" s="215"/>
+      <c r="BL5" s="215"/>
+      <c r="BM5" s="215"/>
+      <c r="BN5" s="215"/>
+      <c r="BO5" s="215"/>
+      <c r="BP5" s="215"/>
     </row>
     <row r="6" spans="1:70">
       <c r="A6"/>
@@ -12507,21 +12510,21 @@
       <c r="AY6" s="49"/>
       <c r="AZ6" s="49"/>
       <c r="BA6" s="49"/>
-      <c r="BB6" s="207"/>
-      <c r="BC6" s="207"/>
-      <c r="BD6" s="207"/>
-      <c r="BE6" s="207"/>
-      <c r="BF6" s="207"/>
-      <c r="BG6" s="207"/>
-      <c r="BH6" s="207"/>
-      <c r="BI6" s="207"/>
-      <c r="BJ6" s="207"/>
-      <c r="BK6" s="207"/>
-      <c r="BL6" s="207"/>
-      <c r="BM6" s="207"/>
-      <c r="BN6" s="207"/>
-      <c r="BO6" s="207"/>
-      <c r="BP6" s="207"/>
+      <c r="BB6" s="215"/>
+      <c r="BC6" s="215"/>
+      <c r="BD6" s="215"/>
+      <c r="BE6" s="215"/>
+      <c r="BF6" s="215"/>
+      <c r="BG6" s="215"/>
+      <c r="BH6" s="215"/>
+      <c r="BI6" s="215"/>
+      <c r="BJ6" s="215"/>
+      <c r="BK6" s="215"/>
+      <c r="BL6" s="215"/>
+      <c r="BM6" s="215"/>
+      <c r="BN6" s="215"/>
+      <c r="BO6" s="215"/>
+      <c r="BP6" s="215"/>
     </row>
     <row r="7" spans="1:70">
       <c r="A7"/>
@@ -12790,20 +12793,20 @@
       <c r="Q13"/>
       <c r="AT13" s="67"/>
       <c r="AU13" s="67"/>
-      <c r="AV13" s="210"/>
-      <c r="AW13" s="210"/>
+      <c r="AV13" s="207"/>
+      <c r="AW13" s="207"/>
       <c r="AX13" s="77"/>
       <c r="AY13" s="78"/>
-      <c r="AZ13" s="211"/>
-      <c r="BA13" s="211"/>
+      <c r="AZ13" s="208"/>
+      <c r="BA13" s="208"/>
       <c r="BB13" s="77"/>
       <c r="BC13" s="141"/>
-      <c r="BD13" s="212"/>
-      <c r="BE13" s="212"/>
+      <c r="BD13" s="209"/>
+      <c r="BE13" s="209"/>
       <c r="BF13" s="71"/>
       <c r="BG13" s="71"/>
-      <c r="BH13" s="212"/>
-      <c r="BI13" s="212"/>
+      <c r="BH13" s="209"/>
+      <c r="BI13" s="209"/>
       <c r="BJ13" s="53"/>
       <c r="BK13" s="53"/>
       <c r="BL13" s="53"/>
@@ -12832,32 +12835,32 @@
       <c r="AH14" s="52"/>
       <c r="AT14" s="67"/>
       <c r="AU14" s="67"/>
-      <c r="AV14" s="210"/>
-      <c r="AW14" s="210"/>
+      <c r="AV14" s="207"/>
+      <c r="AW14" s="207"/>
       <c r="AX14" s="77"/>
       <c r="AY14" s="52"/>
-      <c r="AZ14" s="211"/>
-      <c r="BA14" s="211"/>
+      <c r="AZ14" s="208"/>
+      <c r="BA14" s="208"/>
       <c r="BB14" s="77"/>
       <c r="BC14" s="141"/>
-      <c r="BD14" s="212"/>
-      <c r="BE14" s="212"/>
+      <c r="BD14" s="209"/>
+      <c r="BE14" s="209"/>
       <c r="BF14" s="71"/>
       <c r="BG14" s="71"/>
-      <c r="BH14" s="212"/>
-      <c r="BI14" s="212"/>
+      <c r="BH14" s="209"/>
+      <c r="BI14" s="209"/>
       <c r="BJ14" s="53"/>
       <c r="BK14" s="144" t="s">
         <v>0</v>
       </c>
       <c r="BL14" s="145"/>
-      <c r="BM14" s="213" t="str">
+      <c r="BM14" s="210" t="str">
         <f>'01-Database'!D3</f>
         <v>courseName</v>
       </c>
-      <c r="BN14" s="213"/>
-      <c r="BO14" s="213"/>
-      <c r="BP14" s="213"/>
+      <c r="BN14" s="210"/>
+      <c r="BO14" s="210"/>
+      <c r="BP14" s="210"/>
       <c r="BQ14" s="73"/>
     </row>
     <row r="15" spans="1:70" ht="7.8" customHeight="1">
@@ -12878,20 +12881,20 @@
       <c r="AH15" s="97"/>
       <c r="AT15" s="67"/>
       <c r="AU15" s="67"/>
-      <c r="AV15" s="210"/>
-      <c r="AW15" s="210"/>
+      <c r="AV15" s="207"/>
+      <c r="AW15" s="207"/>
       <c r="AX15" s="77"/>
       <c r="AY15" s="52"/>
-      <c r="AZ15" s="211"/>
-      <c r="BA15" s="211"/>
+      <c r="AZ15" s="208"/>
+      <c r="BA15" s="208"/>
       <c r="BB15" s="77"/>
       <c r="BC15" s="141"/>
-      <c r="BD15" s="212"/>
-      <c r="BE15" s="212"/>
+      <c r="BD15" s="209"/>
+      <c r="BE15" s="209"/>
       <c r="BF15" s="71"/>
       <c r="BG15" s="71"/>
-      <c r="BH15" s="212"/>
-      <c r="BI15" s="212"/>
+      <c r="BH15" s="209"/>
+      <c r="BI15" s="209"/>
       <c r="BJ15" s="53"/>
       <c r="BK15" s="147"/>
       <c r="BL15" s="145"/>
@@ -12919,8 +12922,8 @@
       <c r="AH16" s="97"/>
       <c r="AT16" s="67"/>
       <c r="AU16" s="67"/>
-      <c r="AV16" s="210"/>
-      <c r="AW16" s="210"/>
+      <c r="AV16" s="207"/>
+      <c r="AW16" s="207"/>
       <c r="AX16" s="68"/>
       <c r="AY16" s="52"/>
       <c r="AZ16" s="52"/>
@@ -12938,13 +12941,13 @@
         <v>27</v>
       </c>
       <c r="BL16" s="145"/>
-      <c r="BM16" s="214">
+      <c r="BM16" s="211">
         <f>'01-Database'!F3</f>
         <v>0</v>
       </c>
-      <c r="BN16" s="214"/>
-      <c r="BO16" s="214"/>
-      <c r="BP16" s="214"/>
+      <c r="BN16" s="211"/>
+      <c r="BO16" s="211"/>
+      <c r="BP16" s="211"/>
       <c r="BQ16" s="73"/>
     </row>
     <row r="17" spans="1:69" ht="7.8" customHeight="1">
@@ -12965,8 +12968,8 @@
       <c r="AH17" s="101"/>
       <c r="AT17" s="67"/>
       <c r="AU17" s="67"/>
-      <c r="AV17" s="210"/>
-      <c r="AW17" s="210"/>
+      <c r="AV17" s="207"/>
+      <c r="AW17" s="207"/>
       <c r="AX17" s="52"/>
       <c r="AY17" s="52"/>
       <c r="AZ17" s="67"/>
@@ -13104,13 +13107,13 @@
         <v>3</v>
       </c>
       <c r="BL20" s="146"/>
-      <c r="BM20" s="215" t="str">
+      <c r="BM20" s="212" t="str">
         <f>'01-Database'!Q3</f>
         <v>ชื่อ วิทยากร</v>
       </c>
-      <c r="BN20" s="215"/>
-      <c r="BO20" s="215"/>
-      <c r="BP20" s="215"/>
+      <c r="BN20" s="212"/>
+      <c r="BO20" s="212"/>
+      <c r="BP20" s="212"/>
       <c r="BQ20" s="73"/>
     </row>
     <row r="21" spans="1:69" ht="29.4" customHeight="1">
@@ -13434,13 +13437,13 @@
       <c r="BG30" s="52"/>
       <c r="BH30" s="52"/>
       <c r="BI30" s="102"/>
-      <c r="BJ30" s="208"/>
-      <c r="BK30" s="208"/>
-      <c r="BL30" s="208"/>
-      <c r="BM30" s="208"/>
-      <c r="BN30" s="208"/>
-      <c r="BO30" s="208"/>
-      <c r="BP30" s="208"/>
+      <c r="BJ30" s="206"/>
+      <c r="BK30" s="206"/>
+      <c r="BL30" s="206"/>
+      <c r="BM30" s="206"/>
+      <c r="BN30" s="206"/>
+      <c r="BO30" s="206"/>
+      <c r="BP30" s="206"/>
     </row>
     <row r="31" spans="1:69" ht="15" customHeight="1">
       <c r="A31"/>
@@ -13468,13 +13471,13 @@
       <c r="BG31" s="52"/>
       <c r="BH31" s="52"/>
       <c r="BI31" s="102"/>
-      <c r="BJ31" s="208"/>
-      <c r="BK31" s="208"/>
-      <c r="BL31" s="208"/>
-      <c r="BM31" s="208"/>
-      <c r="BN31" s="208"/>
-      <c r="BO31" s="208"/>
-      <c r="BP31" s="208"/>
+      <c r="BJ31" s="206"/>
+      <c r="BK31" s="206"/>
+      <c r="BL31" s="206"/>
+      <c r="BM31" s="206"/>
+      <c r="BN31" s="206"/>
+      <c r="BO31" s="206"/>
+      <c r="BP31" s="206"/>
     </row>
     <row r="32" spans="1:69" ht="14.25" customHeight="1">
       <c r="A32"/>
@@ -13502,13 +13505,13 @@
       <c r="BG32" s="52"/>
       <c r="BH32" s="52"/>
       <c r="BI32" s="102"/>
-      <c r="BJ32" s="208"/>
-      <c r="BK32" s="208"/>
-      <c r="BL32" s="208"/>
-      <c r="BM32" s="208"/>
-      <c r="BN32" s="208"/>
-      <c r="BO32" s="208"/>
-      <c r="BP32" s="208"/>
+      <c r="BJ32" s="206"/>
+      <c r="BK32" s="206"/>
+      <c r="BL32" s="206"/>
+      <c r="BM32" s="206"/>
+      <c r="BN32" s="206"/>
+      <c r="BO32" s="206"/>
+      <c r="BP32" s="206"/>
     </row>
     <row r="33" spans="1:70" ht="14.25" customHeight="1">
       <c r="A33"/>
@@ -13536,13 +13539,13 @@
       <c r="BG33" s="52"/>
       <c r="BH33" s="52"/>
       <c r="BI33" s="102"/>
-      <c r="BJ33" s="208"/>
-      <c r="BK33" s="208"/>
-      <c r="BL33" s="208"/>
-      <c r="BM33" s="208"/>
-      <c r="BN33" s="208"/>
-      <c r="BO33" s="208"/>
-      <c r="BP33" s="208"/>
+      <c r="BJ33" s="206"/>
+      <c r="BK33" s="206"/>
+      <c r="BL33" s="206"/>
+      <c r="BM33" s="206"/>
+      <c r="BN33" s="206"/>
+      <c r="BO33" s="206"/>
+      <c r="BP33" s="206"/>
     </row>
     <row r="34" spans="1:70" ht="18" customHeight="1">
       <c r="A34"/>
@@ -13570,13 +13573,13 @@
       <c r="BG34" s="52"/>
       <c r="BH34" s="52"/>
       <c r="BI34" s="102"/>
-      <c r="BJ34" s="208"/>
-      <c r="BK34" s="208"/>
-      <c r="BL34" s="208"/>
-      <c r="BM34" s="208"/>
-      <c r="BN34" s="208"/>
-      <c r="BO34" s="208"/>
-      <c r="BP34" s="208"/>
+      <c r="BJ34" s="206"/>
+      <c r="BK34" s="206"/>
+      <c r="BL34" s="206"/>
+      <c r="BM34" s="206"/>
+      <c r="BN34" s="206"/>
+      <c r="BO34" s="206"/>
+      <c r="BP34" s="206"/>
     </row>
     <row r="35" spans="1:70" ht="15">
       <c r="A35"/>
@@ -13604,13 +13607,13 @@
       <c r="BG35" s="52"/>
       <c r="BH35" s="52"/>
       <c r="BI35" s="102"/>
-      <c r="BJ35" s="208"/>
-      <c r="BK35" s="208"/>
-      <c r="BL35" s="208"/>
-      <c r="BM35" s="208"/>
-      <c r="BN35" s="208"/>
-      <c r="BO35" s="208"/>
-      <c r="BP35" s="208"/>
+      <c r="BJ35" s="206"/>
+      <c r="BK35" s="206"/>
+      <c r="BL35" s="206"/>
+      <c r="BM35" s="206"/>
+      <c r="BN35" s="206"/>
+      <c r="BO35" s="206"/>
+      <c r="BP35" s="206"/>
     </row>
     <row r="36" spans="1:70" ht="18.75" customHeight="1">
       <c r="AG36" s="52"/>
@@ -13636,13 +13639,13 @@
       <c r="BG36" s="52"/>
       <c r="BH36" s="52"/>
       <c r="BI36" s="102"/>
-      <c r="BJ36" s="208"/>
-      <c r="BK36" s="208"/>
-      <c r="BL36" s="208"/>
-      <c r="BM36" s="208"/>
-      <c r="BN36" s="208"/>
-      <c r="BO36" s="208"/>
-      <c r="BP36" s="208"/>
+      <c r="BJ36" s="206"/>
+      <c r="BK36" s="206"/>
+      <c r="BL36" s="206"/>
+      <c r="BM36" s="206"/>
+      <c r="BN36" s="206"/>
+      <c r="BO36" s="206"/>
+      <c r="BP36" s="206"/>
     </row>
     <row r="37" spans="1:70" ht="18.75" customHeight="1">
       <c r="AG37" s="52"/>
@@ -13668,13 +13671,13 @@
       <c r="BG37" s="52"/>
       <c r="BH37" s="52"/>
       <c r="BI37" s="102"/>
-      <c r="BJ37" s="208"/>
-      <c r="BK37" s="208"/>
-      <c r="BL37" s="208"/>
-      <c r="BM37" s="208"/>
-      <c r="BN37" s="208"/>
-      <c r="BO37" s="208"/>
-      <c r="BP37" s="208"/>
+      <c r="BJ37" s="206"/>
+      <c r="BK37" s="206"/>
+      <c r="BL37" s="206"/>
+      <c r="BM37" s="206"/>
+      <c r="BN37" s="206"/>
+      <c r="BO37" s="206"/>
+      <c r="BP37" s="206"/>
     </row>
     <row r="38" spans="1:70" ht="18.75" customHeight="1">
       <c r="AG38" s="52"/>
@@ -13700,13 +13703,13 @@
       <c r="BG38" s="84"/>
       <c r="BH38" s="84"/>
       <c r="BI38" s="107"/>
-      <c r="BJ38" s="208"/>
-      <c r="BK38" s="208"/>
-      <c r="BL38" s="208"/>
-      <c r="BM38" s="208"/>
-      <c r="BN38" s="208"/>
-      <c r="BO38" s="208"/>
-      <c r="BP38" s="208"/>
+      <c r="BJ38" s="206"/>
+      <c r="BK38" s="206"/>
+      <c r="BL38" s="206"/>
+      <c r="BM38" s="206"/>
+      <c r="BN38" s="206"/>
+      <c r="BO38" s="206"/>
+      <c r="BP38" s="206"/>
     </row>
     <row r="39" spans="1:70" ht="18.75" customHeight="1">
       <c r="AG39" s="52"/>
@@ -13732,13 +13735,13 @@
       <c r="BG39" s="52"/>
       <c r="BH39" s="52"/>
       <c r="BI39" s="102"/>
-      <c r="BJ39" s="208"/>
-      <c r="BK39" s="208"/>
-      <c r="BL39" s="208"/>
-      <c r="BM39" s="208"/>
-      <c r="BN39" s="208"/>
-      <c r="BO39" s="208"/>
-      <c r="BP39" s="208"/>
+      <c r="BJ39" s="206"/>
+      <c r="BK39" s="206"/>
+      <c r="BL39" s="206"/>
+      <c r="BM39" s="206"/>
+      <c r="BN39" s="206"/>
+      <c r="BO39" s="206"/>
+      <c r="BP39" s="206"/>
     </row>
     <row r="40" spans="1:70" ht="18.75" customHeight="1">
       <c r="AG40" s="52"/>
@@ -13764,13 +13767,13 @@
       <c r="BG40" s="52"/>
       <c r="BH40" s="52"/>
       <c r="BI40" s="102"/>
-      <c r="BJ40" s="208"/>
-      <c r="BK40" s="208"/>
-      <c r="BL40" s="208"/>
-      <c r="BM40" s="208"/>
-      <c r="BN40" s="208"/>
-      <c r="BO40" s="208"/>
-      <c r="BP40" s="208"/>
+      <c r="BJ40" s="206"/>
+      <c r="BK40" s="206"/>
+      <c r="BL40" s="206"/>
+      <c r="BM40" s="206"/>
+      <c r="BN40" s="206"/>
+      <c r="BO40" s="206"/>
+      <c r="BP40" s="206"/>
     </row>
     <row r="41" spans="1:70" ht="18.75" customHeight="1">
       <c r="AG41" s="52"/>
@@ -13796,13 +13799,13 @@
       <c r="BG41" s="52"/>
       <c r="BH41" s="52"/>
       <c r="BI41" s="102"/>
-      <c r="BJ41" s="208"/>
-      <c r="BK41" s="208"/>
-      <c r="BL41" s="208"/>
-      <c r="BM41" s="208"/>
-      <c r="BN41" s="208"/>
-      <c r="BO41" s="208"/>
-      <c r="BP41" s="208"/>
+      <c r="BJ41" s="206"/>
+      <c r="BK41" s="206"/>
+      <c r="BL41" s="206"/>
+      <c r="BM41" s="206"/>
+      <c r="BN41" s="206"/>
+      <c r="BO41" s="206"/>
+      <c r="BP41" s="206"/>
     </row>
     <row r="42" spans="1:70" ht="18.75" customHeight="1">
       <c r="AG42" s="52"/>
@@ -13828,13 +13831,13 @@
       <c r="BG42" s="52"/>
       <c r="BH42" s="52"/>
       <c r="BI42" s="102"/>
-      <c r="BJ42" s="208"/>
-      <c r="BK42" s="208"/>
-      <c r="BL42" s="208"/>
-      <c r="BM42" s="208"/>
-      <c r="BN42" s="208"/>
-      <c r="BO42" s="208"/>
-      <c r="BP42" s="208"/>
+      <c r="BJ42" s="206"/>
+      <c r="BK42" s="206"/>
+      <c r="BL42" s="206"/>
+      <c r="BM42" s="206"/>
+      <c r="BN42" s="206"/>
+      <c r="BO42" s="206"/>
+      <c r="BP42" s="206"/>
     </row>
     <row r="43" spans="1:70" ht="18.75" customHeight="1">
       <c r="AG43" s="52"/>
@@ -13860,13 +13863,13 @@
       <c r="BG43" s="52"/>
       <c r="BH43" s="52"/>
       <c r="BI43" s="52"/>
-      <c r="BJ43" s="209"/>
-      <c r="BK43" s="209"/>
-      <c r="BL43" s="209"/>
-      <c r="BM43" s="209"/>
-      <c r="BN43" s="209"/>
-      <c r="BO43" s="209"/>
-      <c r="BP43" s="209"/>
+      <c r="BJ43" s="213"/>
+      <c r="BK43" s="213"/>
+      <c r="BL43" s="213"/>
+      <c r="BM43" s="213"/>
+      <c r="BN43" s="213"/>
+      <c r="BO43" s="213"/>
+      <c r="BP43" s="213"/>
     </row>
     <row r="44" spans="1:70" ht="18.75" customHeight="1">
       <c r="AG44" s="52"/>
@@ -13892,13 +13895,13 @@
       <c r="BG44" s="52"/>
       <c r="BH44" s="52"/>
       <c r="BI44" s="52"/>
-      <c r="BJ44" s="209"/>
-      <c r="BK44" s="209"/>
-      <c r="BL44" s="209"/>
-      <c r="BM44" s="209"/>
-      <c r="BN44" s="209"/>
-      <c r="BO44" s="209"/>
-      <c r="BP44" s="209"/>
+      <c r="BJ44" s="213"/>
+      <c r="BK44" s="213"/>
+      <c r="BL44" s="213"/>
+      <c r="BM44" s="213"/>
+      <c r="BN44" s="213"/>
+      <c r="BO44" s="213"/>
+      <c r="BP44" s="213"/>
     </row>
     <row r="45" spans="1:70" ht="17.399999999999999">
       <c r="AG45" s="52"/>
@@ -13956,13 +13959,13 @@
       <c r="BG46" s="52"/>
       <c r="BH46" s="52"/>
       <c r="BI46" s="52"/>
-      <c r="BJ46" s="206"/>
-      <c r="BK46" s="206"/>
-      <c r="BL46" s="206"/>
-      <c r="BM46" s="206"/>
-      <c r="BN46" s="206"/>
-      <c r="BO46" s="206"/>
-      <c r="BP46" s="206"/>
+      <c r="BJ46" s="214"/>
+      <c r="BK46" s="214"/>
+      <c r="BL46" s="214"/>
+      <c r="BM46" s="214"/>
+      <c r="BN46" s="214"/>
+      <c r="BO46" s="214"/>
+      <c r="BP46" s="214"/>
     </row>
     <row r="47" spans="1:70" ht="18.75" customHeight="1">
       <c r="AG47" s="52"/>
@@ -13988,13 +13991,13 @@
       <c r="BG47" s="52"/>
       <c r="BH47" s="52"/>
       <c r="BI47" s="52"/>
-      <c r="BJ47" s="206"/>
-      <c r="BK47" s="206"/>
-      <c r="BL47" s="206"/>
-      <c r="BM47" s="206"/>
-      <c r="BN47" s="206"/>
-      <c r="BO47" s="206"/>
-      <c r="BP47" s="206"/>
+      <c r="BJ47" s="214"/>
+      <c r="BK47" s="214"/>
+      <c r="BL47" s="214"/>
+      <c r="BM47" s="214"/>
+      <c r="BN47" s="214"/>
+      <c r="BO47" s="214"/>
+      <c r="BP47" s="214"/>
     </row>
     <row r="48" spans="1:70" ht="18.75" customHeight="1">
       <c r="AG48" s="52"/>
@@ -14020,13 +14023,13 @@
       <c r="BG48" s="52"/>
       <c r="BH48" s="52"/>
       <c r="BI48" s="52"/>
-      <c r="BJ48" s="206"/>
-      <c r="BK48" s="206"/>
-      <c r="BL48" s="206"/>
-      <c r="BM48" s="206"/>
-      <c r="BN48" s="206"/>
-      <c r="BO48" s="206"/>
-      <c r="BP48" s="206"/>
+      <c r="BJ48" s="214"/>
+      <c r="BK48" s="214"/>
+      <c r="BL48" s="214"/>
+      <c r="BM48" s="214"/>
+      <c r="BN48" s="214"/>
+      <c r="BO48" s="214"/>
+      <c r="BP48" s="214"/>
       <c r="BR48" s="156"/>
     </row>
     <row r="49" spans="33:70" ht="18.75" customHeight="1">
@@ -14053,13 +14056,13 @@
       <c r="BG49" s="52"/>
       <c r="BH49" s="52"/>
       <c r="BI49" s="52"/>
-      <c r="BJ49" s="206"/>
-      <c r="BK49" s="206"/>
-      <c r="BL49" s="206"/>
-      <c r="BM49" s="206"/>
-      <c r="BN49" s="206"/>
-      <c r="BO49" s="206"/>
-      <c r="BP49" s="206"/>
+      <c r="BJ49" s="214"/>
+      <c r="BK49" s="214"/>
+      <c r="BL49" s="214"/>
+      <c r="BM49" s="214"/>
+      <c r="BN49" s="214"/>
+      <c r="BO49" s="214"/>
+      <c r="BP49" s="214"/>
       <c r="BR49" s="156"/>
     </row>
     <row r="50" spans="33:70" ht="18.75" customHeight="1">
@@ -14086,13 +14089,13 @@
       <c r="BG50" s="52"/>
       <c r="BH50" s="52"/>
       <c r="BI50" s="52"/>
-      <c r="BJ50" s="206"/>
-      <c r="BK50" s="206"/>
-      <c r="BL50" s="206"/>
-      <c r="BM50" s="206"/>
-      <c r="BN50" s="206"/>
-      <c r="BO50" s="206"/>
-      <c r="BP50" s="206"/>
+      <c r="BJ50" s="214"/>
+      <c r="BK50" s="214"/>
+      <c r="BL50" s="214"/>
+      <c r="BM50" s="214"/>
+      <c r="BN50" s="214"/>
+      <c r="BO50" s="214"/>
+      <c r="BP50" s="214"/>
     </row>
     <row r="51" spans="33:70" ht="18.75" customHeight="1">
       <c r="AG51" s="52"/>
@@ -14118,13 +14121,13 @@
       <c r="BG51" s="52"/>
       <c r="BH51" s="52"/>
       <c r="BI51" s="52"/>
-      <c r="BJ51" s="206"/>
-      <c r="BK51" s="206"/>
-      <c r="BL51" s="206"/>
-      <c r="BM51" s="206"/>
-      <c r="BN51" s="206"/>
-      <c r="BO51" s="206"/>
-      <c r="BP51" s="206"/>
+      <c r="BJ51" s="214"/>
+      <c r="BK51" s="214"/>
+      <c r="BL51" s="214"/>
+      <c r="BM51" s="214"/>
+      <c r="BN51" s="214"/>
+      <c r="BO51" s="214"/>
+      <c r="BP51" s="214"/>
     </row>
     <row r="52" spans="33:70" ht="18.75" customHeight="1">
       <c r="AG52" s="52"/>
@@ -14150,13 +14153,13 @@
       <c r="BG52" s="52"/>
       <c r="BH52" s="52"/>
       <c r="BI52" s="52"/>
-      <c r="BJ52" s="206"/>
-      <c r="BK52" s="206"/>
-      <c r="BL52" s="206"/>
-      <c r="BM52" s="206"/>
-      <c r="BN52" s="206"/>
-      <c r="BO52" s="206"/>
-      <c r="BP52" s="206"/>
+      <c r="BJ52" s="214"/>
+      <c r="BK52" s="214"/>
+      <c r="BL52" s="214"/>
+      <c r="BM52" s="214"/>
+      <c r="BN52" s="214"/>
+      <c r="BO52" s="214"/>
+      <c r="BP52" s="214"/>
     </row>
     <row r="53" spans="33:70" ht="18.75" customHeight="1">
       <c r="AG53" s="52"/>
@@ -14182,13 +14185,13 @@
       <c r="BG53" s="52"/>
       <c r="BH53" s="52"/>
       <c r="BI53" s="52"/>
-      <c r="BJ53" s="206"/>
-      <c r="BK53" s="206"/>
-      <c r="BL53" s="206"/>
-      <c r="BM53" s="206"/>
-      <c r="BN53" s="206"/>
-      <c r="BO53" s="206"/>
-      <c r="BP53" s="206"/>
+      <c r="BJ53" s="214"/>
+      <c r="BK53" s="214"/>
+      <c r="BL53" s="214"/>
+      <c r="BM53" s="214"/>
+      <c r="BN53" s="214"/>
+      <c r="BO53" s="214"/>
+      <c r="BP53" s="214"/>
     </row>
     <row r="54" spans="33:70" ht="18.75" customHeight="1">
       <c r="AG54" s="52"/>
@@ -14214,13 +14217,13 @@
       <c r="BG54" s="52"/>
       <c r="BH54" s="52"/>
       <c r="BI54" s="52"/>
-      <c r="BJ54" s="206"/>
-      <c r="BK54" s="206"/>
-      <c r="BL54" s="206"/>
-      <c r="BM54" s="206"/>
-      <c r="BN54" s="206"/>
-      <c r="BO54" s="206"/>
-      <c r="BP54" s="206"/>
+      <c r="BJ54" s="214"/>
+      <c r="BK54" s="214"/>
+      <c r="BL54" s="214"/>
+      <c r="BM54" s="214"/>
+      <c r="BN54" s="214"/>
+      <c r="BO54" s="214"/>
+      <c r="BP54" s="214"/>
     </row>
     <row r="55" spans="33:70" ht="18.75" customHeight="1">
       <c r="AG55" s="52"/>
@@ -14246,13 +14249,13 @@
       <c r="BG55" s="52"/>
       <c r="BH55" s="52"/>
       <c r="BI55" s="52"/>
-      <c r="BJ55" s="206"/>
-      <c r="BK55" s="206"/>
-      <c r="BL55" s="206"/>
-      <c r="BM55" s="206"/>
-      <c r="BN55" s="206"/>
-      <c r="BO55" s="206"/>
-      <c r="BP55" s="206"/>
+      <c r="BJ55" s="214"/>
+      <c r="BK55" s="214"/>
+      <c r="BL55" s="214"/>
+      <c r="BM55" s="214"/>
+      <c r="BN55" s="214"/>
+      <c r="BO55" s="214"/>
+      <c r="BP55" s="214"/>
     </row>
     <row r="56" spans="33:70" ht="18.75" customHeight="1">
       <c r="AG56" s="52"/>
@@ -14278,13 +14281,13 @@
       <c r="BG56" s="52"/>
       <c r="BH56" s="52"/>
       <c r="BI56" s="52"/>
-      <c r="BJ56" s="206"/>
-      <c r="BK56" s="206"/>
-      <c r="BL56" s="206"/>
-      <c r="BM56" s="206"/>
-      <c r="BN56" s="206"/>
-      <c r="BO56" s="206"/>
-      <c r="BP56" s="206"/>
+      <c r="BJ56" s="214"/>
+      <c r="BK56" s="214"/>
+      <c r="BL56" s="214"/>
+      <c r="BM56" s="214"/>
+      <c r="BN56" s="214"/>
+      <c r="BO56" s="214"/>
+      <c r="BP56" s="214"/>
     </row>
     <row r="57" spans="33:70" ht="18.75" customHeight="1">
       <c r="AG57" s="52"/>
@@ -14310,13 +14313,13 @@
       <c r="BG57" s="52"/>
       <c r="BH57" s="52"/>
       <c r="BI57" s="52"/>
-      <c r="BJ57" s="206"/>
-      <c r="BK57" s="206"/>
-      <c r="BL57" s="206"/>
-      <c r="BM57" s="206"/>
-      <c r="BN57" s="206"/>
-      <c r="BO57" s="206"/>
-      <c r="BP57" s="206"/>
+      <c r="BJ57" s="214"/>
+      <c r="BK57" s="214"/>
+      <c r="BL57" s="214"/>
+      <c r="BM57" s="214"/>
+      <c r="BN57" s="214"/>
+      <c r="BO57" s="214"/>
+      <c r="BP57" s="214"/>
     </row>
     <row r="58" spans="33:70" ht="18.75" customHeight="1">
       <c r="AI58" s="52"/>
@@ -14340,13 +14343,13 @@
       <c r="BG58" s="52"/>
       <c r="BH58" s="52"/>
       <c r="BI58" s="52"/>
-      <c r="BJ58" s="206"/>
-      <c r="BK58" s="206"/>
-      <c r="BL58" s="206"/>
-      <c r="BM58" s="206"/>
-      <c r="BN58" s="206"/>
-      <c r="BO58" s="206"/>
-      <c r="BP58" s="206"/>
+      <c r="BJ58" s="214"/>
+      <c r="BK58" s="214"/>
+      <c r="BL58" s="214"/>
+      <c r="BM58" s="214"/>
+      <c r="BN58" s="214"/>
+      <c r="BO58" s="214"/>
+      <c r="BP58" s="214"/>
     </row>
     <row r="59" spans="33:70" ht="18.75" customHeight="1">
       <c r="AI59" s="52"/>
@@ -14370,13 +14373,13 @@
       <c r="BG59" s="52"/>
       <c r="BH59" s="52"/>
       <c r="BI59" s="52"/>
-      <c r="BJ59" s="206"/>
-      <c r="BK59" s="206"/>
-      <c r="BL59" s="206"/>
-      <c r="BM59" s="206"/>
-      <c r="BN59" s="206"/>
-      <c r="BO59" s="206"/>
-      <c r="BP59" s="206"/>
+      <c r="BJ59" s="214"/>
+      <c r="BK59" s="214"/>
+      <c r="BL59" s="214"/>
+      <c r="BM59" s="214"/>
+      <c r="BN59" s="214"/>
+      <c r="BO59" s="214"/>
+      <c r="BP59" s="214"/>
     </row>
     <row r="60" spans="33:70" ht="18.75" customHeight="1">
       <c r="AI60" s="52"/>
@@ -14400,13 +14403,13 @@
       <c r="BG60" s="52"/>
       <c r="BH60" s="52"/>
       <c r="BI60" s="52"/>
-      <c r="BJ60" s="206"/>
-      <c r="BK60" s="206"/>
-      <c r="BL60" s="206"/>
-      <c r="BM60" s="206"/>
-      <c r="BN60" s="206"/>
-      <c r="BO60" s="206"/>
-      <c r="BP60" s="206"/>
+      <c r="BJ60" s="214"/>
+      <c r="BK60" s="214"/>
+      <c r="BL60" s="214"/>
+      <c r="BM60" s="214"/>
+      <c r="BN60" s="214"/>
+      <c r="BO60" s="214"/>
+      <c r="BP60" s="214"/>
     </row>
     <row r="61" spans="33:70" ht="17.399999999999999">
       <c r="AI61" s="52"/>
@@ -14961,28 +14964,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1" sort="0" autoFilter="0" selectUnlockedCells="1"/>
   <mergeCells count="38">
-    <mergeCell ref="BJ34:BP34"/>
-    <mergeCell ref="AV13:AW17"/>
-    <mergeCell ref="AZ13:BA15"/>
-    <mergeCell ref="BD13:BE15"/>
-    <mergeCell ref="BH13:BI15"/>
-    <mergeCell ref="BM14:BP14"/>
-    <mergeCell ref="BM16:BP16"/>
-    <mergeCell ref="BM20:BP20"/>
-    <mergeCell ref="BJ30:BP30"/>
-    <mergeCell ref="BJ31:BP31"/>
-    <mergeCell ref="BJ32:BP32"/>
-    <mergeCell ref="BJ33:BP33"/>
-    <mergeCell ref="BJ43:BP43"/>
-    <mergeCell ref="BJ44:BP44"/>
-    <mergeCell ref="BJ46:BP46"/>
-    <mergeCell ref="BJ47:BP47"/>
-    <mergeCell ref="BJ35:BP35"/>
-    <mergeCell ref="BJ36:BP36"/>
-    <mergeCell ref="BJ37:BP37"/>
-    <mergeCell ref="BJ38:BP38"/>
-    <mergeCell ref="BJ39:BP39"/>
-    <mergeCell ref="BJ40:BP40"/>
     <mergeCell ref="BJ60:BP60"/>
     <mergeCell ref="BB3:BP6"/>
     <mergeCell ref="BJ54:BP54"/>
@@ -14999,6 +14980,28 @@
     <mergeCell ref="BJ53:BP53"/>
     <mergeCell ref="BJ41:BP41"/>
     <mergeCell ref="BJ42:BP42"/>
+    <mergeCell ref="BJ43:BP43"/>
+    <mergeCell ref="BJ44:BP44"/>
+    <mergeCell ref="BJ46:BP46"/>
+    <mergeCell ref="BJ47:BP47"/>
+    <mergeCell ref="BJ35:BP35"/>
+    <mergeCell ref="BJ36:BP36"/>
+    <mergeCell ref="BJ37:BP37"/>
+    <mergeCell ref="BJ38:BP38"/>
+    <mergeCell ref="BJ39:BP39"/>
+    <mergeCell ref="BJ40:BP40"/>
+    <mergeCell ref="BJ34:BP34"/>
+    <mergeCell ref="AV13:AW17"/>
+    <mergeCell ref="AZ13:BA15"/>
+    <mergeCell ref="BD13:BE15"/>
+    <mergeCell ref="BH13:BI15"/>
+    <mergeCell ref="BM14:BP14"/>
+    <mergeCell ref="BM16:BP16"/>
+    <mergeCell ref="BM20:BP20"/>
+    <mergeCell ref="BJ30:BP30"/>
+    <mergeCell ref="BJ31:BP31"/>
+    <mergeCell ref="BJ32:BP32"/>
+    <mergeCell ref="BJ33:BP33"/>
   </mergeCells>
   <pageMargins left="0.37" right="0.31" top="0.41" bottom="0.32" header="0.2" footer="0.3"/>
   <pageSetup paperSize="9" scale="42" fitToHeight="0" orientation="portrait" r:id="rId1"/>

</xml_diff>